<commit_message>
docs: adicionando requisitos não funcionais
</commit_message>
<xml_diff>
--- a/docs/01 - Levantamento de Requisitos/Matriz de Rastreabilidade de Requisitos.xlsx
+++ b/docs/01 - Levantamento de Requisitos/Matriz de Rastreabilidade de Requisitos.xlsx
@@ -1,17 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\OneDrive\Documentos\SCRIPTS\HTML E CSS\projetos\PsiSoft\docs\01 - Levantamento de Requisitos\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="17256" windowHeight="5796"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Matriz de Rastreabilidade de Re" sheetId="1" r:id="rId5"/>
+    <sheet name="Matriz de Rastreabilidade de Re" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="143">
   <si>
     <t>ID</t>
   </si>
@@ -410,22 +418,68 @@
   </si>
   <si>
     <t>Requisito RD-P01</t>
+  </si>
+  <si>
+    <t>RN-07</t>
+  </si>
+  <si>
+    <t>RN-08</t>
+  </si>
+  <si>
+    <t>Entrevista Psicóloga</t>
+  </si>
+  <si>
+    <t>Transcrição com IA: Após uma sessão acontecer, o sistema deve transcrever automaticamente e gerar o prontuário da sessão.</t>
+  </si>
+  <si>
+    <t>Entrevista Psicologo.pdf</t>
+  </si>
+  <si>
+    <t>Respostas 1 e 2</t>
+  </si>
+  <si>
+    <t>Conformidade com o CFP: A estrutura do prontuário eletrônico deve seguir rigorosamente as informações obrigatórias exigidas pela Resolução CFP n° 001/2009.</t>
+  </si>
+  <si>
+    <t>resolucao2009-01.pdf</t>
+  </si>
+  <si>
+    <t>Resolução CFP N° 001/2009</t>
+  </si>
+  <si>
+    <t>Regras Gerais do Prontuário</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -434,35 +488,42 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -470,7 +531,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -660,23 +721,26 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:E35"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="83.75"/>
-    <col customWidth="1" min="3" max="3" width="82.25"/>
-    <col customWidth="1" min="4" max="4" width="91.75"/>
-    <col customWidth="1" min="5" max="5" width="31.0"/>
+    <col min="2" max="2" width="112.5546875" customWidth="1"/>
+    <col min="3" max="3" width="82.21875" customWidth="1"/>
+    <col min="4" max="4" width="91.77734375" customWidth="1"/>
+    <col min="5" max="5" width="31" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -693,7 +757,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -710,7 +774,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
@@ -727,7 +791,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
@@ -744,7 +808,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>20</v>
       </c>
@@ -761,7 +825,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>25</v>
       </c>
@@ -778,7 +842,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>30</v>
       </c>
@@ -795,7 +859,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>35</v>
       </c>
@@ -812,7 +876,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>38</v>
       </c>
@@ -829,7 +893,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>43</v>
       </c>
@@ -846,7 +910,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>46</v>
       </c>
@@ -863,7 +927,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>49</v>
       </c>
@@ -880,7 +944,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>52</v>
       </c>
@@ -897,7 +961,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>57</v>
       </c>
@@ -914,7 +978,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>60</v>
       </c>
@@ -931,7 +995,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>63</v>
       </c>
@@ -948,7 +1012,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>66</v>
       </c>
@@ -965,7 +1029,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>69</v>
       </c>
@@ -982,7 +1046,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>74</v>
       </c>
@@ -999,7 +1063,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>79</v>
       </c>
@@ -1016,7 +1080,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>82</v>
       </c>
@@ -1033,7 +1097,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>87</v>
       </c>
@@ -1050,7 +1114,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>92</v>
       </c>
@@ -1067,7 +1131,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>95</v>
       </c>
@@ -1084,7 +1148,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>98</v>
       </c>
@@ -1101,7 +1165,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>103</v>
       </c>
@@ -1118,7 +1182,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>108</v>
       </c>
@@ -1135,7 +1199,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>113</v>
       </c>
@@ -1152,7 +1216,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>118</v>
       </c>
@@ -1169,7 +1233,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:5" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>121</v>
       </c>
@@ -1186,58 +1250,93 @@
         <v>123</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="1" t="s">
+    <row r="31" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="B33" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="C31" s="1" t="s">
+      <c r="C33" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="D31" s="1" t="s">
+      <c r="D33" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="E31" s="1" t="s">
+      <c r="E33" s="1" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="1" t="s">
+    <row r="34" spans="1:5" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B34" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="C34" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="D32" s="1" t="s">
+      <c r="D34" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="E32" s="1" t="s">
+      <c r="E34" s="1" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="1" t="s">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B35" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="C33" s="2" t="s">
+      <c r="C35" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D33" s="1" t="s">
+      <c r="D35" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E33" s="1" t="s">
+      <c r="E35" s="1" t="s">
         <v>132</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>